<commit_message>
Improve unmatched DS3 handling: borrow GPS or drop
Unmatched DS3 rows (band resights with no DS1 group match) are now
handled by checking if the route exists anywhere in DS1 on the same date:
  • Route found in DS1 → borrow GPS from that DS1 entry, keep the row
    with a comment noting coordinates are approximate
  • Route not in DS1 at all → drop the row (band info without any
    location is not useful)

Also fixes substring route matching so DS3 "Pavilion Key" correctly
resolves to DS1 "Everglades City to Pavilion Key".

Result: 103 rows, all with GPS, 0 partial-location warnings.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Databases/Database3/Output/2017/db3_2017_FINAL.xlsx
+++ b/Databases/Database3/Output/2017/db3_2017_FINAL.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Clean_Data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Removed_Rows" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Summary_Report" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clean_Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Removed_Rows" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary_Report" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7288,8 +7288,12 @@
           <t>Pavilion Key</t>
         </is>
       </c>
-      <c r="F103" t="inlineStr"/>
-      <c r="G103" t="inlineStr"/>
+      <c r="F103" t="n">
+        <v>25.694949</v>
+      </c>
+      <c r="G103" t="n">
+        <v>-81.348572</v>
+      </c>
       <c r="H103" t="n">
         <v>1</v>
       </c>
@@ -7314,7 +7318,7 @@
       </c>
       <c r="N103" t="inlineStr">
         <is>
-          <t>Missing lower left foot.  Have pictures.</t>
+          <t>Missing lower left foot.  Have pictures. | GPS approx: no group match in DS1 — coordinates from DS1 group 4 at same route/date</t>
         </is>
       </c>
       <c r="O103" t="inlineStr">
@@ -7347,8 +7351,12 @@
           <t>Pavilion Key</t>
         </is>
       </c>
-      <c r="F104" t="inlineStr"/>
-      <c r="G104" t="inlineStr"/>
+      <c r="F104" t="n">
+        <v>25.694949</v>
+      </c>
+      <c r="G104" t="n">
+        <v>-81.348572</v>
+      </c>
       <c r="H104" t="n">
         <v>1</v>
       </c>
@@ -7369,7 +7377,7 @@
       </c>
       <c r="N104" t="inlineStr">
         <is>
-          <t>May be missing flag from upper right leg. Other bands match the PIPL Sid saw here 2 years ago. Have pictures.</t>
+          <t>May be missing flag from upper right leg. Other bands match the PIPL Sid saw here 2 years ago. Have pictures. | GPS approx: no group match in DS1 — coordinates from DS1 group 4 at same route/date</t>
         </is>
       </c>
       <c r="O104" t="inlineStr">
@@ -7429,7 +7437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -7456,7 +7464,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-20 13:28</t>
+          <t>2026-04-21 11:54</t>
         </is>
       </c>
     </row>
@@ -7717,32 +7725,16 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">  unique_id 102</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Missing: Latitude, Longitude</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  unique_id 103</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Missing: Latitude, Longitude</t>
-        </is>
-      </c>
+          <t xml:space="preserve">  None</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>